<commit_message>
Agregar busqueda de gobernadores y corregir limite de TPM de Groq
Suma columna de gobernador/jefe de gobierno (busqueda, extraccion, CSV,
Excel, comparacion) y deja placeholders vacios en maestro.json para
verificar a mano. Corrige un HTTP 413 real de Groq (12.000 TPM) acotando
el contexto por entidad en vez de dejarlo crecer sin limite; validado con
dos corridas reales.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Autoridades de Min. Seg y FFSS - Fed y Prov (Listado y Fuentes).xlsx
+++ b/Autoridades de Min. Seg y FFSS - Fed y Prov (Listado y Fuentes).xlsx
@@ -9,18 +9,20 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17970" windowHeight="8340" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17970" windowHeight="8340" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Jurisdicciones Provinciales y C" sheetId="1" r:id="rId1"/>
     <sheet name="maestro_20260716" sheetId="2" r:id="rId2"/>
+    <sheet name="autoridades_20260716" sheetId="3" r:id="rId3"/>
+    <sheet name="autoridades_20260716_2" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="386">
   <si>
     <t>Jurisdicción</t>
   </si>
@@ -973,6 +975,327 @@
   </si>
   <si>
     <t>Comisario General Mauricio Zabala</t>
+  </si>
+  <si>
+    <t>Gobernador</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/normativa/nacional/decreto-383-2025-414065/texto</t>
+  </si>
+  <si>
+    <t>Policia Federal Argentina (PFA)</t>
+  </si>
+  <si>
+    <t>NO ENCONTRADO</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/gendarmeria</t>
+  </si>
+  <si>
+    <t>Gendarmeria Nacional Argentina (GNA)</t>
+  </si>
+  <si>
+    <t>Claudio Miguel Brilloni</t>
+  </si>
+  <si>
+    <t>Aníbal Ariel Bronzetti</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/noticias/se-conformo-la-nueva-plana-mayor-de-la-prefectura-naval-argentina</t>
+  </si>
+  <si>
+    <t>Prefectura Naval Argentina (PNA)</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/psa</t>
+  </si>
+  <si>
+    <t>Policia de Seguridad Aeroportuaria (PSA)</t>
+  </si>
+  <si>
+    <t>Dr. Carlos Tonelli Banfi</t>
+  </si>
+  <si>
+    <t>Valeria Endrek</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/servicio-penitenciario-federal</t>
+  </si>
+  <si>
+    <t>Servicio Penitenciario Federal (SPF)</t>
+  </si>
+  <si>
+    <t>Lic. Fernando Martínez</t>
+  </si>
+  <si>
+    <t>Horacio Rodríguez Larreta (Jefe de Gobierno)</t>
+  </si>
+  <si>
+    <t>https://buenosaires.gob.ar/gcaba_historico/jefe-de-gobierno</t>
+  </si>
+  <si>
+    <t>Cordoba</t>
+  </si>
+  <si>
+    <t>Martín Llaryora (Gobernador)</t>
+  </si>
+  <si>
+    <t>Pablo Quinteros (Ministro de Seguridad)</t>
+  </si>
+  <si>
+    <t>https://www.cba.gov.ar/estructura-del-gobierno</t>
+  </si>
+  <si>
+    <t>Marcelo Marin</t>
+  </si>
+  <si>
+    <t>Federico Cisneros</t>
+  </si>
+  <si>
+    <t>Maximiliano Nicolás Pullaro (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.santafe.gov.ar/index.php/content/download/224123/1174128</t>
+  </si>
+  <si>
+    <t>https://prensa.mendoza.gob.ar/mercedes-rus-presento-en-la-legislatura-el-presupuesto-2026-nuestro-objetivo-es-ambicioso-y-estamos-avanzando-con-decision-firmeza-y-resultados</t>
+  </si>
+  <si>
+    <t>Tucuman</t>
+  </si>
+  <si>
+    <t>Osvaldo Francisco Jaldo (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.tucuman.gob.ar/gobernador</t>
+  </si>
+  <si>
+    <t>Gustavo Saenz (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.salta.gob.ar</t>
+  </si>
+  <si>
+    <t>Carlos Ariel Gil Urquiola (Secretario de Seguridad Pública)</t>
+  </si>
+  <si>
+    <t>https://hacienda.jujuy.gob.ar/designacion-del-nuevo-secretario-de-seguridad-publica</t>
+  </si>
+  <si>
+    <t>Entre Rios</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/seguridad/transparencia/autoridades-personal</t>
+  </si>
+  <si>
+    <t>Juan Pablo Valdés (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://munired.mcypcorrientes.gob.ar/gobierno-de-la-provincia-de-corrientes</t>
+  </si>
+  <si>
+    <t>https://gobierno.misiones.gob.ar/guia-de-autoridades</t>
+  </si>
+  <si>
+    <t>Leandro Zdero (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://chaco.gob.ar</t>
+  </si>
+  <si>
+    <t>Neuquen</t>
+  </si>
+  <si>
+    <t>https://www.neuqueninforma.gob.ar/noticias/2026/03/10/255534-una-nueva-etapa-en-el-fortalecimiento-de-la-seguridad-publica</t>
+  </si>
+  <si>
+    <t>Tomás Díaz Pérez</t>
+  </si>
+  <si>
+    <t>Walter San Martín</t>
+  </si>
+  <si>
+    <t>Rio Negro</t>
+  </si>
+  <si>
+    <t>Alberto Weretilneck (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://rionegro.gov.ar</t>
+  </si>
+  <si>
+    <t>NO ENCONTRADO (Ministro de Seguridad)</t>
+  </si>
+  <si>
+    <t>https://jusnoticias.juschubut.gov.ar/el-stj-recibio-al-ministro-de-seguridad-y-a-las-nuevas-autoridades-de-la-policia-del-chubut</t>
+  </si>
+  <si>
+    <t>César Brandt</t>
+  </si>
+  <si>
+    <t>Juan Cruz Campos</t>
+  </si>
+  <si>
+    <t>Claudio Orlando Vidal (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.santacruz.gob.ar/gobierno/autoridades</t>
+  </si>
+  <si>
+    <t>Gustavo Adrián Melella (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.tierradelfuego.gob.ar/autoridades-gob</t>
+  </si>
+  <si>
+    <t>Marcelo Rego (Gobernador)</t>
+  </si>
+  <si>
+    <t>Gustavo Fariña (Secretario de Seguridad y Orden Público)</t>
+  </si>
+  <si>
+    <t>https://contenido.sanjuan.gob.ar/index.php?option=com_k2&amp;view=item&amp;id=1343%3Aasumio-el-nuevo-subjefe-de-policia</t>
+  </si>
+  <si>
+    <t>Luis Walter Ma</t>
+  </si>
+  <si>
+    <t>José Luis Morales</t>
+  </si>
+  <si>
+    <t>Claudio Poggi (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/noticias/el-mandato-de-los-argentinos-es-terminar-con-el-pasado-y-volver-abrazar-las-ideas-que</t>
+  </si>
+  <si>
+    <t>Raúl Jalil (Gobernador)</t>
+  </si>
+  <si>
+    <t>Alberto Natella (Ministro de Gobierno, Seguridad y Justicia)</t>
+  </si>
+  <si>
+    <t>https://portal.catamarca.gob.ar/</t>
+  </si>
+  <si>
+    <t>Crio. Gral. Marcelo Ulises Córdoba</t>
+  </si>
+  <si>
+    <t>Crio. Gral. Víctor Hugo Sánchez</t>
+  </si>
+  <si>
+    <t>Sergio Ziliotto (Gobernador)</t>
+  </si>
+  <si>
+    <t>Horacio Esteban Di Nápoli (Ministro de Seguridad)</t>
+  </si>
+  <si>
+    <t>https://www.lapampa.gob.ar</t>
+  </si>
+  <si>
+    <t>Gildo Insfrán (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.formosa.gob.ar</t>
+  </si>
+  <si>
+    <t>C.P.N. Atilio Chara (Ministro de Gobierno, Seguridad y Culto)</t>
+  </si>
+  <si>
+    <t>http://www.boletinsde.gov.ar</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/prefecturanaval</t>
+  </si>
+  <si>
+    <t>Guillermo José Giménez Pérez</t>
+  </si>
+  <si>
+    <t>Alejandro Paulo Annichini</t>
+  </si>
+  <si>
+    <t>Carlos Tonelli Banfi</t>
+  </si>
+  <si>
+    <t>Fernando Martínez</t>
+  </si>
+  <si>
+    <t>NO ENCONTRADO (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.mendoza.gob.ar</t>
+  </si>
+  <si>
+    <t>https://www.tucuman.gob.ar</t>
+  </si>
+  <si>
+    <t>Gustavo Sáenz (Gobernador)</t>
+  </si>
+  <si>
+    <t>Gaspar Solá Usandivaras (Ministro de Seguridad y Justicia)</t>
+  </si>
+  <si>
+    <t>José Alberto Ibarra</t>
+  </si>
+  <si>
+    <t>Adriana Herrera</t>
+  </si>
+  <si>
+    <t>https://seguridad.jujuy.gob.ar</t>
+  </si>
+  <si>
+    <t>https://www.entrerios.gov.ar/boletin/calendario/Boletin/2026/Marzo/26-03-26.pdf</t>
+  </si>
+  <si>
+    <t>Claudio Omar GONZALEZ</t>
+  </si>
+  <si>
+    <t>Leandro Cesar Zdero (Gobernador)</t>
+  </si>
+  <si>
+    <t>Andres Garcia</t>
+  </si>
+  <si>
+    <t>Javier Pedro Prodromos (Ministro de Seguridad)</t>
+  </si>
+  <si>
+    <t>Diego Agüero</t>
+  </si>
+  <si>
+    <t>Marcelo Orrego (Gobernador)</t>
+  </si>
+  <si>
+    <t>Enrique Delgado (Secretario de Seguridad y Orden Público)</t>
+  </si>
+  <si>
+    <t>https://diputadossanjuan.gob.ar/prensa/11495-asumio-el-nuevo-secretario-de-seguridad-y-orden-publico</t>
+  </si>
+  <si>
+    <t>Luis Walter Martínez</t>
+  </si>
+  <si>
+    <t>Ricardo Quintela (Gobernador)</t>
+  </si>
+  <si>
+    <t>https://www.legislaturasconectadas.gob.ar/Prensa/Quintela-Madera-asumieron-como-gobernador-y-vicegobernadora-de-La-Rioja/4485</t>
+  </si>
+  <si>
+    <t>https://policiadecatamarca.gob.ar/noticias/autoridades/principal</t>
+  </si>
+  <si>
+    <t>Víctor Hugo Sánchez</t>
+  </si>
+  <si>
+    <t>https://www.argentina.gob.ar/noticias/frederic-se-reunio-con-el-ministro-de-seguridad-de-la-pampa</t>
+  </si>
+  <si>
+    <t>Jorge Abel González (Ministro de Gobierno, Justicia, Seguridad y Trabajo)</t>
+  </si>
+  <si>
+    <t>https://www.formosa.gob.ar/mingobierno</t>
+  </si>
+  <si>
+    <t>Atilio Chara (Ministro de Gobierno, Seguridad y Culto)</t>
   </si>
 </sst>
 </file>
@@ -1044,12 +1367,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1064,7 +1393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1098,27 +1427,12 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1143,13 +1457,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Jurisdicciones Provinciales y C-style" pivot="0" count="4">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2882,4 +3212,1410 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="152.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D2" t="s">
+        <v>280</v>
+      </c>
+      <c r="E2" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I2" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" t="s">
+        <v>283</v>
+      </c>
+      <c r="E3" t="s">
+        <v>284</v>
+      </c>
+      <c r="F3" t="s">
+        <v>285</v>
+      </c>
+      <c r="G3" t="s">
+        <v>286</v>
+      </c>
+      <c r="I3" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" t="s">
+        <v>287</v>
+      </c>
+      <c r="E4" t="s">
+        <v>288</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I4" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D5" t="s">
+        <v>289</v>
+      </c>
+      <c r="E5" t="s">
+        <v>290</v>
+      </c>
+      <c r="F5" t="s">
+        <v>291</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="I5" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D6" t="s">
+        <v>293</v>
+      </c>
+      <c r="E6" t="s">
+        <v>294</v>
+      </c>
+      <c r="F6" t="s">
+        <v>295</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I6" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>282</v>
+      </c>
+      <c r="C7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>282</v>
+      </c>
+      <c r="G7" t="s">
+        <v>282</v>
+      </c>
+      <c r="I7" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" t="s">
+        <v>282</v>
+      </c>
+      <c r="D8" t="s">
+        <v>297</v>
+      </c>
+      <c r="F8" t="s">
+        <v>282</v>
+      </c>
+      <c r="G8" t="s">
+        <v>282</v>
+      </c>
+      <c r="I8" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B9" t="s">
+        <v>299</v>
+      </c>
+      <c r="C9" t="s">
+        <v>300</v>
+      </c>
+      <c r="D9" t="s">
+        <v>301</v>
+      </c>
+      <c r="F9" t="s">
+        <v>302</v>
+      </c>
+      <c r="G9" t="s">
+        <v>303</v>
+      </c>
+      <c r="I9" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D10" t="s">
+        <v>305</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I10" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>282</v>
+      </c>
+      <c r="C11" t="s">
+        <v>216</v>
+      </c>
+      <c r="D11" t="s">
+        <v>306</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I11" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>307</v>
+      </c>
+      <c r="B12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C12" t="s">
+        <v>282</v>
+      </c>
+      <c r="D12" t="s">
+        <v>309</v>
+      </c>
+      <c r="F12" t="s">
+        <v>282</v>
+      </c>
+      <c r="G12" t="s">
+        <v>282</v>
+      </c>
+      <c r="I12" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>310</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D13" t="s">
+        <v>311</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I13" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" t="s">
+        <v>282</v>
+      </c>
+      <c r="C14" t="s">
+        <v>312</v>
+      </c>
+      <c r="D14" t="s">
+        <v>313</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I14" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>314</v>
+      </c>
+      <c r="B15" t="s">
+        <v>282</v>
+      </c>
+      <c r="C15" t="s">
+        <v>282</v>
+      </c>
+      <c r="D15" t="s">
+        <v>315</v>
+      </c>
+      <c r="F15" t="s">
+        <v>282</v>
+      </c>
+      <c r="G15" t="s">
+        <v>282</v>
+      </c>
+      <c r="I15" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D16" t="s">
+        <v>317</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I16" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" t="s">
+        <v>226</v>
+      </c>
+      <c r="D17" t="s">
+        <v>318</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I17" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I18" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>321</v>
+      </c>
+      <c r="B19" t="s">
+        <v>282</v>
+      </c>
+      <c r="C19" t="s">
+        <v>244</v>
+      </c>
+      <c r="D19" t="s">
+        <v>322</v>
+      </c>
+      <c r="F19" t="s">
+        <v>323</v>
+      </c>
+      <c r="G19" t="s">
+        <v>324</v>
+      </c>
+      <c r="I19" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>325</v>
+      </c>
+      <c r="B20" t="s">
+        <v>326</v>
+      </c>
+      <c r="C20" t="s">
+        <v>282</v>
+      </c>
+      <c r="D20" t="s">
+        <v>327</v>
+      </c>
+      <c r="F20" t="s">
+        <v>282</v>
+      </c>
+      <c r="G20" t="s">
+        <v>282</v>
+      </c>
+      <c r="I20" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21" t="s">
+        <v>282</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="D21" t="s">
+        <v>329</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="I21" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D22" t="s">
+        <v>333</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I22" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>161</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D23" t="s">
+        <v>335</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I23" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>140</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="D24" t="s">
+        <v>338</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="I24" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D25" t="s">
+        <v>342</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I25" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" t="s">
+        <v>282</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D26" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I26" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="D27" t="s">
+        <v>345</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="I27" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="C28" t="s">
+        <v>349</v>
+      </c>
+      <c r="D28" t="s">
+        <v>350</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G28" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I28" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>120</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D29" t="s">
+        <v>352</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I29" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" t="s">
+        <v>282</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>353</v>
+      </c>
+      <c r="D30" t="s">
+        <v>354</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I30" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="113.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E2" t="s">
+        <v>281</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I2" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" t="s">
+        <v>283</v>
+      </c>
+      <c r="E3" t="s">
+        <v>284</v>
+      </c>
+      <c r="F3" t="s">
+        <v>285</v>
+      </c>
+      <c r="G3" t="s">
+        <v>286</v>
+      </c>
+      <c r="I3" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D4" t="s">
+        <v>355</v>
+      </c>
+      <c r="E4" t="s">
+        <v>288</v>
+      </c>
+      <c r="F4" t="s">
+        <v>356</v>
+      </c>
+      <c r="G4" t="s">
+        <v>357</v>
+      </c>
+      <c r="I4" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D5" t="s">
+        <v>289</v>
+      </c>
+      <c r="E5" t="s">
+        <v>290</v>
+      </c>
+      <c r="F5" t="s">
+        <v>358</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="I5" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D6" t="s">
+        <v>293</v>
+      </c>
+      <c r="E6" t="s">
+        <v>294</v>
+      </c>
+      <c r="F6" t="s">
+        <v>359</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I6" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>360</v>
+      </c>
+      <c r="C7" t="s">
+        <v>204</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>282</v>
+      </c>
+      <c r="G7" t="s">
+        <v>282</v>
+      </c>
+      <c r="I7" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" t="s">
+        <v>282</v>
+      </c>
+      <c r="D8" t="s">
+        <v>297</v>
+      </c>
+      <c r="F8" t="s">
+        <v>282</v>
+      </c>
+      <c r="G8" t="s">
+        <v>282</v>
+      </c>
+      <c r="I8" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B9" t="s">
+        <v>299</v>
+      </c>
+      <c r="C9" t="s">
+        <v>300</v>
+      </c>
+      <c r="D9" t="s">
+        <v>301</v>
+      </c>
+      <c r="F9" t="s">
+        <v>302</v>
+      </c>
+      <c r="G9" t="s">
+        <v>303</v>
+      </c>
+      <c r="I9" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D10" t="s">
+        <v>305</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I10" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>360</v>
+      </c>
+      <c r="C11" t="s">
+        <v>216</v>
+      </c>
+      <c r="D11" t="s">
+        <v>361</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I11" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>307</v>
+      </c>
+      <c r="B12" t="s">
+        <v>308</v>
+      </c>
+      <c r="C12" t="s">
+        <v>282</v>
+      </c>
+      <c r="D12" t="s">
+        <v>362</v>
+      </c>
+      <c r="F12" t="s">
+        <v>282</v>
+      </c>
+      <c r="G12" t="s">
+        <v>282</v>
+      </c>
+      <c r="I12" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>364</v>
+      </c>
+      <c r="D13" t="s">
+        <v>311</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>366</v>
+      </c>
+      <c r="I13" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" t="s">
+        <v>360</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="D14" t="s">
+        <v>367</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I14" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>314</v>
+      </c>
+      <c r="B15" t="s">
+        <v>282</v>
+      </c>
+      <c r="C15" t="s">
+        <v>282</v>
+      </c>
+      <c r="D15" t="s">
+        <v>368</v>
+      </c>
+      <c r="F15" t="s">
+        <v>369</v>
+      </c>
+      <c r="G15" t="s">
+        <v>282</v>
+      </c>
+      <c r="I15" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D16" t="s">
+        <v>317</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I16" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" t="s">
+        <v>226</v>
+      </c>
+      <c r="D17" t="s">
+        <v>318</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I17" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>370</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I18" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>321</v>
+      </c>
+      <c r="B19" t="s">
+        <v>282</v>
+      </c>
+      <c r="C19" t="s">
+        <v>244</v>
+      </c>
+      <c r="D19" t="s">
+        <v>322</v>
+      </c>
+      <c r="F19" t="s">
+        <v>323</v>
+      </c>
+      <c r="G19" t="s">
+        <v>324</v>
+      </c>
+      <c r="I19" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>325</v>
+      </c>
+      <c r="B20" t="s">
+        <v>326</v>
+      </c>
+      <c r="C20" t="s">
+        <v>248</v>
+      </c>
+      <c r="D20" t="s">
+        <v>108</v>
+      </c>
+      <c r="F20" t="s">
+        <v>282</v>
+      </c>
+      <c r="G20" t="s">
+        <v>282</v>
+      </c>
+      <c r="I20" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21" t="s">
+        <v>282</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="D21" t="s">
+        <v>174</v>
+      </c>
+      <c r="F21" t="s">
+        <v>371</v>
+      </c>
+      <c r="G21" t="s">
+        <v>173</v>
+      </c>
+      <c r="I21" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="C22" t="s">
+        <v>372</v>
+      </c>
+      <c r="D22" t="s">
+        <v>333</v>
+      </c>
+      <c r="F22" t="s">
+        <v>373</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I22" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>161</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D23" t="s">
+        <v>335</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I23" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>140</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="C24" t="s">
+        <v>375</v>
+      </c>
+      <c r="D24" t="s">
+        <v>376</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="I24" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D25" t="s">
+        <v>342</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I25" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="D26" t="s">
+        <v>379</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I26" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="D27" t="s">
+        <v>380</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G27" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="I27" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>348</v>
+      </c>
+      <c r="C28" t="s">
+        <v>257</v>
+      </c>
+      <c r="D28" t="s">
+        <v>382</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G28" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I28" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>120</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="C29" t="s">
+        <v>383</v>
+      </c>
+      <c r="D29" t="s">
+        <v>384</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I29" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" t="s">
+        <v>360</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="D30" t="s">
+        <v>354</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I30" s="11">
+        <v>46219</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerar Excel desde maestro tras las correcciones de hoy
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Autoridades de Min. Seg y FFSS - Fed y Prov (Listado y Fuentes).xlsx
+++ b/Autoridades de Min. Seg y FFSS - Fed y Prov (Listado y Fuentes).xlsx
@@ -9,20 +9,22 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17970" windowHeight="8340" firstSheet="1" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17970" windowHeight="8340" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Jurisdicciones Provinciales y C" sheetId="1" r:id="rId1"/>
     <sheet name="maestro_20260716" sheetId="2" r:id="rId2"/>
     <sheet name="autoridades_20260716" sheetId="3" r:id="rId3"/>
     <sheet name="autoridades_20260716_2" sheetId="4" r:id="rId4"/>
+    <sheet name="maestro_20260717" sheetId="5" r:id="rId5"/>
+    <sheet name="maestro_20260717_2" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="392">
   <si>
     <t>Jurisdicción</t>
   </si>
@@ -1296,6 +1298,24 @@
   </si>
   <si>
     <t>Atilio Chara (Ministro de Gobierno, Seguridad y Culto)</t>
+  </si>
+  <si>
+    <t>Comisionado General María Lorena Anderch</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (Jefe de Gobierno)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (Gobernador)</t>
+  </si>
+  <si>
+    <t>Nicolás Avellaneda (Ministro de Seguridad y Justicia)</t>
+  </si>
+  <si>
+    <t>Fernando Monguillot (Ministro de Seguridad)</t>
+  </si>
+  <si>
+    <t>Bernardo José Herrera (Ministro de Gobierno, Seguridad y Culto)</t>
   </si>
 </sst>
 </file>
@@ -4618,4 +4638,1380 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="127.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G2" t="s">
+        <v>180</v>
+      </c>
+      <c r="I2" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G3" t="s">
+        <v>184</v>
+      </c>
+      <c r="I3" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F4" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" t="s">
+        <v>188</v>
+      </c>
+      <c r="I4" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G5" t="s">
+        <v>386</v>
+      </c>
+      <c r="I5" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="E6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" t="s">
+        <v>195</v>
+      </c>
+      <c r="G6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I6" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B7" t="s">
+        <v>387</v>
+      </c>
+      <c r="C7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E7" t="s">
+        <v>200</v>
+      </c>
+      <c r="F7" t="s">
+        <v>201</v>
+      </c>
+      <c r="G7" t="s">
+        <v>202</v>
+      </c>
+      <c r="I7" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" t="s">
+        <v>388</v>
+      </c>
+      <c r="C8" t="s">
+        <v>204</v>
+      </c>
+      <c r="E8" t="s">
+        <v>205</v>
+      </c>
+      <c r="F8" t="s">
+        <v>206</v>
+      </c>
+      <c r="G8" t="s">
+        <v>207</v>
+      </c>
+      <c r="I8" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>388</v>
+      </c>
+      <c r="C9" t="s">
+        <v>208</v>
+      </c>
+      <c r="E9" t="s">
+        <v>209</v>
+      </c>
+      <c r="F9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G9" t="s">
+        <v>211</v>
+      </c>
+      <c r="I9" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
+        <v>388</v>
+      </c>
+      <c r="C10" t="s">
+        <v>212</v>
+      </c>
+      <c r="E10" t="s">
+        <v>213</v>
+      </c>
+      <c r="F10" t="s">
+        <v>214</v>
+      </c>
+      <c r="G10" t="s">
+        <v>215</v>
+      </c>
+      <c r="I10" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>388</v>
+      </c>
+      <c r="C11" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G11" t="s">
+        <v>218</v>
+      </c>
+      <c r="I11" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>388</v>
+      </c>
+      <c r="C12" t="s">
+        <v>219</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" t="s">
+        <v>220</v>
+      </c>
+      <c r="G12" t="s">
+        <v>221</v>
+      </c>
+      <c r="I12" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" t="s">
+        <v>388</v>
+      </c>
+      <c r="C13" t="s">
+        <v>222</v>
+      </c>
+      <c r="E13" t="s">
+        <v>223</v>
+      </c>
+      <c r="F13" t="s">
+        <v>224</v>
+      </c>
+      <c r="G13" t="s">
+        <v>225</v>
+      </c>
+      <c r="I13" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" t="s">
+        <v>388</v>
+      </c>
+      <c r="C14" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" t="s">
+        <v>227</v>
+      </c>
+      <c r="G14" t="s">
+        <v>228</v>
+      </c>
+      <c r="I14" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>388</v>
+      </c>
+      <c r="C15" t="s">
+        <v>229</v>
+      </c>
+      <c r="E15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" t="s">
+        <v>230</v>
+      </c>
+      <c r="G15" t="s">
+        <v>231</v>
+      </c>
+      <c r="I15" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" t="s">
+        <v>388</v>
+      </c>
+      <c r="C16" t="s">
+        <v>232</v>
+      </c>
+      <c r="E16" t="s">
+        <v>74</v>
+      </c>
+      <c r="F16" t="s">
+        <v>233</v>
+      </c>
+      <c r="G16" t="s">
+        <v>234</v>
+      </c>
+      <c r="I16" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" t="s">
+        <v>388</v>
+      </c>
+      <c r="C17" t="s">
+        <v>235</v>
+      </c>
+      <c r="E17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
+        <v>236</v>
+      </c>
+      <c r="G17" t="s">
+        <v>237</v>
+      </c>
+      <c r="I17" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C18" t="s">
+        <v>238</v>
+      </c>
+      <c r="E18" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" t="s">
+        <v>239</v>
+      </c>
+      <c r="G18" t="s">
+        <v>240</v>
+      </c>
+      <c r="I18" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" t="s">
+        <v>388</v>
+      </c>
+      <c r="C19" t="s">
+        <v>241</v>
+      </c>
+      <c r="E19" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" t="s">
+        <v>242</v>
+      </c>
+      <c r="G19" t="s">
+        <v>243</v>
+      </c>
+      <c r="I19" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" t="s">
+        <v>388</v>
+      </c>
+      <c r="C20" t="s">
+        <v>244</v>
+      </c>
+      <c r="E20" t="s">
+        <v>245</v>
+      </c>
+      <c r="F20" t="s">
+        <v>246</v>
+      </c>
+      <c r="G20" t="s">
+        <v>247</v>
+      </c>
+      <c r="I20" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
+        <v>388</v>
+      </c>
+      <c r="C21" t="s">
+        <v>248</v>
+      </c>
+      <c r="E21" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21" t="s">
+        <v>249</v>
+      </c>
+      <c r="G21" t="s">
+        <v>250</v>
+      </c>
+      <c r="I21" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C22" t="s">
+        <v>251</v>
+      </c>
+      <c r="E22" t="s">
+        <v>116</v>
+      </c>
+      <c r="F22" t="s">
+        <v>252</v>
+      </c>
+      <c r="G22" t="s">
+        <v>253</v>
+      </c>
+      <c r="I22" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" t="s">
+        <v>388</v>
+      </c>
+      <c r="C23" t="s">
+        <v>254</v>
+      </c>
+      <c r="E23" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G23" t="s">
+        <v>256</v>
+      </c>
+      <c r="I23" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>388</v>
+      </c>
+      <c r="C24" t="s">
+        <v>257</v>
+      </c>
+      <c r="E24" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" t="s">
+        <v>258</v>
+      </c>
+      <c r="G24" t="s">
+        <v>259</v>
+      </c>
+      <c r="I24" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" t="s">
+        <v>388</v>
+      </c>
+      <c r="C25" t="s">
+        <v>260</v>
+      </c>
+      <c r="E25" t="s">
+        <v>136</v>
+      </c>
+      <c r="F25" t="s">
+        <v>261</v>
+      </c>
+      <c r="G25" t="s">
+        <v>262</v>
+      </c>
+      <c r="I25" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>140</v>
+      </c>
+      <c r="B26" t="s">
+        <v>388</v>
+      </c>
+      <c r="C26" t="s">
+        <v>263</v>
+      </c>
+      <c r="E26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F26" t="s">
+        <v>264</v>
+      </c>
+      <c r="G26" t="s">
+        <v>265</v>
+      </c>
+      <c r="I26" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B27" t="s">
+        <v>388</v>
+      </c>
+      <c r="C27" t="s">
+        <v>266</v>
+      </c>
+      <c r="E27" t="s">
+        <v>150</v>
+      </c>
+      <c r="F27" t="s">
+        <v>267</v>
+      </c>
+      <c r="G27" t="s">
+        <v>268</v>
+      </c>
+      <c r="I27" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>154</v>
+      </c>
+      <c r="B28" t="s">
+        <v>388</v>
+      </c>
+      <c r="C28" t="s">
+        <v>269</v>
+      </c>
+      <c r="E28" t="s">
+        <v>157</v>
+      </c>
+      <c r="F28" t="s">
+        <v>270</v>
+      </c>
+      <c r="G28" t="s">
+        <v>271</v>
+      </c>
+      <c r="I28" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>161</v>
+      </c>
+      <c r="B29" t="s">
+        <v>388</v>
+      </c>
+      <c r="C29" t="s">
+        <v>272</v>
+      </c>
+      <c r="E29" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" t="s">
+        <v>273</v>
+      </c>
+      <c r="G29" t="s">
+        <v>274</v>
+      </c>
+      <c r="I29" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>168</v>
+      </c>
+      <c r="B30" t="s">
+        <v>388</v>
+      </c>
+      <c r="C30" t="s">
+        <v>275</v>
+      </c>
+      <c r="E30" t="s">
+        <v>276</v>
+      </c>
+      <c r="F30" t="s">
+        <v>277</v>
+      </c>
+      <c r="G30" t="s">
+        <v>278</v>
+      </c>
+      <c r="I30" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="42.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="127.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F2" t="s">
+        <v>179</v>
+      </c>
+      <c r="G2" t="s">
+        <v>180</v>
+      </c>
+      <c r="I2" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G3" t="s">
+        <v>184</v>
+      </c>
+      <c r="I3" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F4" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" t="s">
+        <v>188</v>
+      </c>
+      <c r="I4" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F5" t="s">
+        <v>191</v>
+      </c>
+      <c r="G5" t="s">
+        <v>386</v>
+      </c>
+      <c r="I5" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="E6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" t="s">
+        <v>195</v>
+      </c>
+      <c r="G6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I6" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B7" t="s">
+        <v>387</v>
+      </c>
+      <c r="C7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E7" t="s">
+        <v>200</v>
+      </c>
+      <c r="F7" t="s">
+        <v>201</v>
+      </c>
+      <c r="G7" t="s">
+        <v>202</v>
+      </c>
+      <c r="I7" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" t="s">
+        <v>388</v>
+      </c>
+      <c r="C8" t="s">
+        <v>204</v>
+      </c>
+      <c r="E8" t="s">
+        <v>205</v>
+      </c>
+      <c r="F8" t="s">
+        <v>206</v>
+      </c>
+      <c r="G8" t="s">
+        <v>207</v>
+      </c>
+      <c r="I8" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>388</v>
+      </c>
+      <c r="C9" t="s">
+        <v>208</v>
+      </c>
+      <c r="E9" t="s">
+        <v>209</v>
+      </c>
+      <c r="F9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G9" t="s">
+        <v>211</v>
+      </c>
+      <c r="I9" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
+        <v>388</v>
+      </c>
+      <c r="C10" t="s">
+        <v>212</v>
+      </c>
+      <c r="E10" t="s">
+        <v>213</v>
+      </c>
+      <c r="F10" t="s">
+        <v>214</v>
+      </c>
+      <c r="G10" t="s">
+        <v>215</v>
+      </c>
+      <c r="I10" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>388</v>
+      </c>
+      <c r="C11" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G11" t="s">
+        <v>218</v>
+      </c>
+      <c r="I11" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>388</v>
+      </c>
+      <c r="C12" t="s">
+        <v>219</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" t="s">
+        <v>220</v>
+      </c>
+      <c r="G12" t="s">
+        <v>221</v>
+      </c>
+      <c r="I12" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" t="s">
+        <v>388</v>
+      </c>
+      <c r="C13" t="s">
+        <v>222</v>
+      </c>
+      <c r="E13" t="s">
+        <v>223</v>
+      </c>
+      <c r="F13" t="s">
+        <v>224</v>
+      </c>
+      <c r="G13" t="s">
+        <v>225</v>
+      </c>
+      <c r="I13" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" t="s">
+        <v>388</v>
+      </c>
+      <c r="C14" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" t="s">
+        <v>227</v>
+      </c>
+      <c r="G14" t="s">
+        <v>228</v>
+      </c>
+      <c r="I14" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>388</v>
+      </c>
+      <c r="C15" t="s">
+        <v>389</v>
+      </c>
+      <c r="E15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" t="s">
+        <v>230</v>
+      </c>
+      <c r="G15" t="s">
+        <v>231</v>
+      </c>
+      <c r="I15" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" t="s">
+        <v>388</v>
+      </c>
+      <c r="C16" t="s">
+        <v>232</v>
+      </c>
+      <c r="E16" t="s">
+        <v>74</v>
+      </c>
+      <c r="F16" t="s">
+        <v>233</v>
+      </c>
+      <c r="G16" t="s">
+        <v>234</v>
+      </c>
+      <c r="I16" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" t="s">
+        <v>388</v>
+      </c>
+      <c r="C17" t="s">
+        <v>235</v>
+      </c>
+      <c r="E17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
+        <v>236</v>
+      </c>
+      <c r="G17" t="s">
+        <v>237</v>
+      </c>
+      <c r="I17" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" t="s">
+        <v>388</v>
+      </c>
+      <c r="C18" t="s">
+        <v>238</v>
+      </c>
+      <c r="E18" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" t="s">
+        <v>239</v>
+      </c>
+      <c r="G18" t="s">
+        <v>240</v>
+      </c>
+      <c r="I18" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B19" t="s">
+        <v>388</v>
+      </c>
+      <c r="C19" t="s">
+        <v>241</v>
+      </c>
+      <c r="E19" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" t="s">
+        <v>242</v>
+      </c>
+      <c r="G19" t="s">
+        <v>243</v>
+      </c>
+      <c r="I19" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" t="s">
+        <v>388</v>
+      </c>
+      <c r="C20" t="s">
+        <v>244</v>
+      </c>
+      <c r="E20" t="s">
+        <v>245</v>
+      </c>
+      <c r="F20" t="s">
+        <v>246</v>
+      </c>
+      <c r="G20" t="s">
+        <v>247</v>
+      </c>
+      <c r="I20" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s">
+        <v>388</v>
+      </c>
+      <c r="C21" t="s">
+        <v>248</v>
+      </c>
+      <c r="E21" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21" t="s">
+        <v>249</v>
+      </c>
+      <c r="G21" t="s">
+        <v>250</v>
+      </c>
+      <c r="I21" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" t="s">
+        <v>388</v>
+      </c>
+      <c r="C22" t="s">
+        <v>390</v>
+      </c>
+      <c r="E22" t="s">
+        <v>116</v>
+      </c>
+      <c r="F22" t="s">
+        <v>252</v>
+      </c>
+      <c r="G22" t="s">
+        <v>253</v>
+      </c>
+      <c r="I22" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" t="s">
+        <v>388</v>
+      </c>
+      <c r="C23" t="s">
+        <v>254</v>
+      </c>
+      <c r="E23" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G23" t="s">
+        <v>256</v>
+      </c>
+      <c r="I23" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>388</v>
+      </c>
+      <c r="C24" t="s">
+        <v>257</v>
+      </c>
+      <c r="E24" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" t="s">
+        <v>258</v>
+      </c>
+      <c r="G24" t="s">
+        <v>259</v>
+      </c>
+      <c r="I24" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" t="s">
+        <v>388</v>
+      </c>
+      <c r="C25" t="s">
+        <v>260</v>
+      </c>
+      <c r="E25" t="s">
+        <v>136</v>
+      </c>
+      <c r="F25" t="s">
+        <v>261</v>
+      </c>
+      <c r="G25" t="s">
+        <v>262</v>
+      </c>
+      <c r="I25" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>140</v>
+      </c>
+      <c r="B26" t="s">
+        <v>388</v>
+      </c>
+      <c r="C26" t="s">
+        <v>263</v>
+      </c>
+      <c r="E26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F26" t="s">
+        <v>264</v>
+      </c>
+      <c r="G26" t="s">
+        <v>265</v>
+      </c>
+      <c r="I26" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>147</v>
+      </c>
+      <c r="B27" t="s">
+        <v>388</v>
+      </c>
+      <c r="C27" t="s">
+        <v>266</v>
+      </c>
+      <c r="E27" t="s">
+        <v>150</v>
+      </c>
+      <c r="F27" t="s">
+        <v>267</v>
+      </c>
+      <c r="G27" t="s">
+        <v>268</v>
+      </c>
+      <c r="I27" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>154</v>
+      </c>
+      <c r="B28" t="s">
+        <v>388</v>
+      </c>
+      <c r="C28" t="s">
+        <v>391</v>
+      </c>
+      <c r="E28" t="s">
+        <v>157</v>
+      </c>
+      <c r="F28" t="s">
+        <v>270</v>
+      </c>
+      <c r="G28" t="s">
+        <v>271</v>
+      </c>
+      <c r="I28" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>161</v>
+      </c>
+      <c r="B29" t="s">
+        <v>388</v>
+      </c>
+      <c r="C29" t="s">
+        <v>272</v>
+      </c>
+      <c r="E29" t="s">
+        <v>164</v>
+      </c>
+      <c r="F29" t="s">
+        <v>273</v>
+      </c>
+      <c r="G29" t="s">
+        <v>274</v>
+      </c>
+      <c r="I29" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>168</v>
+      </c>
+      <c r="B30" t="s">
+        <v>388</v>
+      </c>
+      <c r="C30" t="s">
+        <v>275</v>
+      </c>
+      <c r="E30" t="s">
+        <v>276</v>
+      </c>
+      <c r="F30" t="s">
+        <v>277</v>
+      </c>
+      <c r="G30" t="s">
+        <v>278</v>
+      </c>
+      <c r="I30" s="11">
+        <v>46135</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>